<commit_message>
completed yyc ProcedureClinics mapping
</commit_message>
<xml_diff>
--- a/procedure_lookup_project.xlsx
+++ b/procedure_lookup_project.xlsx
@@ -13874,24 +13874,24 @@
     </row>
     <row r="524">
       <c r="A524" s="1">
-        <v>615.0</v>
+        <v>616.0</v>
       </c>
       <c r="B524" s="1">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
       <c r="C524" s="1">
         <v>9.0</v>
       </c>
       <c r="D524" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="1">
-        <v>616.0</v>
+        <v>617.0</v>
       </c>
       <c r="B525" s="1">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="C525" s="1">
         <v>9.0</v>
@@ -13902,7 +13902,7 @@
     </row>
     <row r="526">
       <c r="A526" s="1">
-        <v>617.0</v>
+        <v>618.0</v>
       </c>
       <c r="B526" s="1">
         <v>32.0</v>
@@ -13911,29 +13911,29 @@
         <v>9.0</v>
       </c>
       <c r="D526" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="1">
-        <v>618.0</v>
+        <v>619.0</v>
       </c>
       <c r="B527" s="1">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
       <c r="C527" s="1">
         <v>9.0</v>
       </c>
       <c r="D527" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="1">
-        <v>619.0</v>
+        <v>620.0</v>
       </c>
       <c r="B528" s="1">
-        <v>33.0</v>
+        <v>34.0</v>
       </c>
       <c r="C528" s="1">
         <v>9.0</v>
@@ -13944,10 +13944,10 @@
     </row>
     <row r="529">
       <c r="A529" s="1">
-        <v>620.0</v>
+        <v>621.0</v>
       </c>
       <c r="B529" s="1">
-        <v>34.0</v>
+        <v>35.0</v>
       </c>
       <c r="C529" s="1">
         <v>9.0</v>
@@ -13958,10 +13958,10 @@
     </row>
     <row r="530">
       <c r="A530" s="1">
-        <v>621.0</v>
+        <v>622.0</v>
       </c>
       <c r="B530" s="1">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
       <c r="C530" s="1">
         <v>9.0</v>
@@ -13972,10 +13972,10 @@
     </row>
     <row r="531">
       <c r="A531" s="1">
-        <v>622.0</v>
+        <v>623.0</v>
       </c>
       <c r="B531" s="1">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="C531" s="1">
         <v>9.0</v>
@@ -13986,10 +13986,10 @@
     </row>
     <row r="532">
       <c r="A532" s="1">
-        <v>623.0</v>
+        <v>624.0</v>
       </c>
       <c r="B532" s="1">
-        <v>37.0</v>
+        <v>38.0</v>
       </c>
       <c r="C532" s="1">
         <v>9.0</v>
@@ -14000,10 +14000,10 @@
     </row>
     <row r="533">
       <c r="A533" s="1">
-        <v>624.0</v>
+        <v>625.0</v>
       </c>
       <c r="B533" s="1">
-        <v>38.0</v>
+        <v>40.0</v>
       </c>
       <c r="C533" s="1">
         <v>9.0</v>
@@ -14014,10 +14014,10 @@
     </row>
     <row r="534">
       <c r="A534" s="1">
-        <v>625.0</v>
+        <v>626.0</v>
       </c>
       <c r="B534" s="1">
-        <v>40.0</v>
+        <v>41.0</v>
       </c>
       <c r="C534" s="1">
         <v>9.0</v>
@@ -14028,10 +14028,10 @@
     </row>
     <row r="535">
       <c r="A535" s="1">
-        <v>626.0</v>
+        <v>627.0</v>
       </c>
       <c r="B535" s="1">
-        <v>41.0</v>
+        <v>42.0</v>
       </c>
       <c r="C535" s="1">
         <v>9.0</v>
@@ -14039,13 +14039,16 @@
       <c r="D535" s="1">
         <v>1.0</v>
       </c>
+      <c r="E535" s="1" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="1">
-        <v>627.0</v>
+        <v>628.0</v>
       </c>
       <c r="B536" s="1">
-        <v>42.0</v>
+        <v>57.0</v>
       </c>
       <c r="C536" s="1">
         <v>9.0</v>
@@ -14054,15 +14057,15 @@
         <v>1.0</v>
       </c>
       <c r="E536" s="1" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="1">
-        <v>628.0</v>
+        <v>629.0</v>
       </c>
       <c r="B537" s="1">
-        <v>57.0</v>
+        <v>58.0</v>
       </c>
       <c r="C537" s="1">
         <v>9.0</v>
@@ -14076,10 +14079,10 @@
     </row>
     <row r="538">
       <c r="A538" s="1">
-        <v>629.0</v>
+        <v>630.0</v>
       </c>
       <c r="B538" s="1">
-        <v>58.0</v>
+        <v>59.0</v>
       </c>
       <c r="C538" s="1">
         <v>9.0</v>
@@ -14093,10 +14096,10 @@
     </row>
     <row r="539">
       <c r="A539" s="1">
-        <v>630.0</v>
+        <v>631.0</v>
       </c>
       <c r="B539" s="1">
-        <v>59.0</v>
+        <v>60.0</v>
       </c>
       <c r="C539" s="1">
         <v>9.0</v>
@@ -14110,10 +14113,10 @@
     </row>
     <row r="540">
       <c r="A540" s="1">
-        <v>631.0</v>
+        <v>632.0</v>
       </c>
       <c r="B540" s="1">
-        <v>60.0</v>
+        <v>63.0</v>
       </c>
       <c r="C540" s="1">
         <v>9.0</v>
@@ -14122,15 +14125,15 @@
         <v>1.0</v>
       </c>
       <c r="E540" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="1">
-        <v>632.0</v>
+        <v>633.0</v>
       </c>
       <c r="B541" s="1">
-        <v>63.0</v>
+        <v>64.0</v>
       </c>
       <c r="C541" s="1">
         <v>9.0</v>
@@ -14139,21 +14142,21 @@
         <v>1.0</v>
       </c>
       <c r="E541" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="1">
-        <v>633.0</v>
+        <v>634.0</v>
       </c>
       <c r="B542" s="1">
-        <v>64.0</v>
+        <v>65.0</v>
       </c>
       <c r="C542" s="1">
         <v>9.0</v>
       </c>
       <c r="D542" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E542" s="1" t="s">
         <v>424</v>
@@ -14161,10 +14164,10 @@
     </row>
     <row r="543">
       <c r="A543" s="1">
-        <v>634.0</v>
+        <v>635.0</v>
       </c>
       <c r="B543" s="1">
-        <v>65.0</v>
+        <v>111.0</v>
       </c>
       <c r="C543" s="1">
         <v>9.0</v>
@@ -14172,36 +14175,36 @@
       <c r="D543" s="1">
         <v>2.0</v>
       </c>
-      <c r="E543" s="1" t="s">
-        <v>424</v>
-      </c>
     </row>
     <row r="544">
       <c r="A544" s="1">
-        <v>635.0</v>
+        <v>636.0</v>
       </c>
       <c r="B544" s="1">
-        <v>111.0</v>
+        <v>66.0</v>
       </c>
       <c r="C544" s="1">
         <v>9.0</v>
       </c>
       <c r="D544" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
+      </c>
+      <c r="E544" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="1">
-        <v>636.0</v>
+        <v>637.0</v>
       </c>
       <c r="B545" s="1">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
       <c r="C545" s="1">
         <v>9.0</v>
       </c>
       <c r="D545" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E545" s="1" t="s">
         <v>427</v>
@@ -14209,10 +14212,10 @@
     </row>
     <row r="546">
       <c r="A546" s="1">
-        <v>637.0</v>
+        <v>638.0</v>
       </c>
       <c r="B546" s="1">
-        <v>67.0</v>
+        <v>70.0</v>
       </c>
       <c r="C546" s="1">
         <v>9.0</v>
@@ -14221,15 +14224,15 @@
         <v>2.0</v>
       </c>
       <c r="E546" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="1">
-        <v>638.0</v>
+        <v>639.0</v>
       </c>
       <c r="B547" s="1">
-        <v>70.0</v>
+        <v>77.0</v>
       </c>
       <c r="C547" s="1">
         <v>9.0</v>
@@ -14243,10 +14246,10 @@
     </row>
     <row r="548">
       <c r="A548" s="1">
-        <v>639.0</v>
+        <v>640.0</v>
       </c>
       <c r="B548" s="1">
-        <v>77.0</v>
+        <v>82.0</v>
       </c>
       <c r="C548" s="1">
         <v>9.0</v>
@@ -14260,27 +14263,24 @@
     </row>
     <row r="549">
       <c r="A549" s="1">
-        <v>640.0</v>
+        <v>641.0</v>
       </c>
       <c r="B549" s="1">
-        <v>82.0</v>
+        <v>1.0</v>
       </c>
       <c r="C549" s="1">
-        <v>9.0</v>
+        <v>11.0</v>
       </c>
       <c r="D549" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="E549" s="1" t="s">
-        <v>428</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="1">
-        <v>641.0</v>
+        <v>642.0</v>
       </c>
       <c r="B550" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C550" s="1">
         <v>11.0</v>
@@ -14291,10 +14291,10 @@
     </row>
     <row r="551">
       <c r="A551" s="1">
-        <v>642.0</v>
+        <v>643.0</v>
       </c>
       <c r="B551" s="1">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="C551" s="1">
         <v>11.0</v>
@@ -14305,10 +14305,10 @@
     </row>
     <row r="552">
       <c r="A552" s="1">
-        <v>643.0</v>
+        <v>644.0</v>
       </c>
       <c r="B552" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C552" s="1">
         <v>11.0</v>
@@ -14319,10 +14319,10 @@
     </row>
     <row r="553">
       <c r="A553" s="1">
-        <v>644.0</v>
+        <v>645.0</v>
       </c>
       <c r="B553" s="1">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C553" s="1">
         <v>11.0</v>
@@ -14333,10 +14333,10 @@
     </row>
     <row r="554">
       <c r="A554" s="1">
-        <v>645.0</v>
+        <v>646.0</v>
       </c>
       <c r="B554" s="1">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="C554" s="1">
         <v>11.0</v>
@@ -14347,10 +14347,10 @@
     </row>
     <row r="555">
       <c r="A555" s="1">
-        <v>646.0</v>
+        <v>647.0</v>
       </c>
       <c r="B555" s="1">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="C555" s="1">
         <v>11.0</v>
@@ -14361,10 +14361,10 @@
     </row>
     <row r="556">
       <c r="A556" s="1">
-        <v>647.0</v>
+        <v>648.0</v>
       </c>
       <c r="B556" s="1">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="C556" s="1">
         <v>11.0</v>
@@ -14375,10 +14375,10 @@
     </row>
     <row r="557">
       <c r="A557" s="1">
-        <v>648.0</v>
+        <v>649.0</v>
       </c>
       <c r="B557" s="1">
-        <v>8.0</v>
+        <v>9.0</v>
       </c>
       <c r="C557" s="1">
         <v>11.0</v>
@@ -14389,10 +14389,10 @@
     </row>
     <row r="558">
       <c r="A558" s="1">
-        <v>649.0</v>
+        <v>650.0</v>
       </c>
       <c r="B558" s="1">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
       <c r="C558" s="1">
         <v>11.0</v>
@@ -14403,10 +14403,10 @@
     </row>
     <row r="559">
       <c r="A559" s="1">
-        <v>650.0</v>
+        <v>651.0</v>
       </c>
       <c r="B559" s="1">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
       <c r="C559" s="1">
         <v>11.0</v>
@@ -14417,10 +14417,10 @@
     </row>
     <row r="560">
       <c r="A560" s="1">
-        <v>651.0</v>
+        <v>652.0</v>
       </c>
       <c r="B560" s="1">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="C560" s="1">
         <v>11.0</v>
@@ -14431,10 +14431,10 @@
     </row>
     <row r="561">
       <c r="A561" s="1">
-        <v>652.0</v>
+        <v>653.0</v>
       </c>
       <c r="B561" s="1">
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="C561" s="1">
         <v>11.0</v>
@@ -14445,10 +14445,10 @@
     </row>
     <row r="562">
       <c r="A562" s="1">
-        <v>653.0</v>
+        <v>654.0</v>
       </c>
       <c r="B562" s="1">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
       <c r="C562" s="1">
         <v>11.0</v>
@@ -14459,10 +14459,10 @@
     </row>
     <row r="563">
       <c r="A563" s="1">
-        <v>654.0</v>
+        <v>655.0</v>
       </c>
       <c r="B563" s="1">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="C563" s="1">
         <v>11.0</v>
@@ -14473,10 +14473,10 @@
     </row>
     <row r="564">
       <c r="A564" s="1">
-        <v>655.0</v>
+        <v>656.0</v>
       </c>
       <c r="B564" s="1">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C564" s="1">
         <v>11.0</v>
@@ -14487,10 +14487,10 @@
     </row>
     <row r="565">
       <c r="A565" s="1">
-        <v>656.0</v>
+        <v>657.0</v>
       </c>
       <c r="B565" s="1">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
       <c r="C565" s="1">
         <v>11.0</v>
@@ -14501,10 +14501,10 @@
     </row>
     <row r="566">
       <c r="A566" s="1">
-        <v>657.0</v>
+        <v>658.0</v>
       </c>
       <c r="B566" s="1">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
       <c r="C566" s="1">
         <v>11.0</v>
@@ -14515,10 +14515,10 @@
     </row>
     <row r="567">
       <c r="A567" s="1">
-        <v>658.0</v>
+        <v>659.0</v>
       </c>
       <c r="B567" s="1">
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="C567" s="1">
         <v>11.0</v>
@@ -14529,10 +14529,10 @@
     </row>
     <row r="568">
       <c r="A568" s="1">
-        <v>659.0</v>
+        <v>660.0</v>
       </c>
       <c r="B568" s="1">
-        <v>19.0</v>
+        <v>20.0</v>
       </c>
       <c r="C568" s="1">
         <v>11.0</v>
@@ -14543,10 +14543,10 @@
     </row>
     <row r="569">
       <c r="A569" s="1">
-        <v>660.0</v>
+        <v>661.0</v>
       </c>
       <c r="B569" s="1">
-        <v>20.0</v>
+        <v>21.0</v>
       </c>
       <c r="C569" s="1">
         <v>11.0</v>
@@ -14557,10 +14557,10 @@
     </row>
     <row r="570">
       <c r="A570" s="1">
-        <v>661.0</v>
+        <v>662.0</v>
       </c>
       <c r="B570" s="1">
-        <v>21.0</v>
+        <v>22.0</v>
       </c>
       <c r="C570" s="1">
         <v>11.0</v>
@@ -14571,10 +14571,10 @@
     </row>
     <row r="571">
       <c r="A571" s="1">
-        <v>662.0</v>
+        <v>663.0</v>
       </c>
       <c r="B571" s="1">
-        <v>22.0</v>
+        <v>23.0</v>
       </c>
       <c r="C571" s="1">
         <v>11.0</v>
@@ -14585,10 +14585,10 @@
     </row>
     <row r="572">
       <c r="A572" s="1">
-        <v>663.0</v>
+        <v>664.0</v>
       </c>
       <c r="B572" s="1">
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="C572" s="1">
         <v>11.0</v>
@@ -14599,10 +14599,10 @@
     </row>
     <row r="573">
       <c r="A573" s="1">
-        <v>664.0</v>
+        <v>665.0</v>
       </c>
       <c r="B573" s="1">
-        <v>24.0</v>
+        <v>25.0</v>
       </c>
       <c r="C573" s="1">
         <v>11.0</v>
@@ -14613,10 +14613,10 @@
     </row>
     <row r="574">
       <c r="A574" s="1">
-        <v>665.0</v>
+        <v>666.0</v>
       </c>
       <c r="B574" s="1">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="C574" s="1">
         <v>11.0</v>
@@ -14627,10 +14627,10 @@
     </row>
     <row r="575">
       <c r="A575" s="1">
-        <v>666.0</v>
+        <v>667.0</v>
       </c>
       <c r="B575" s="1">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
       <c r="C575" s="1">
         <v>11.0</v>
@@ -14641,10 +14641,10 @@
     </row>
     <row r="576">
       <c r="A576" s="1">
-        <v>667.0</v>
+        <v>668.0</v>
       </c>
       <c r="B576" s="1">
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
       <c r="C576" s="1">
         <v>11.0</v>
@@ -14655,10 +14655,10 @@
     </row>
     <row r="577">
       <c r="A577" s="1">
-        <v>668.0</v>
+        <v>669.0</v>
       </c>
       <c r="B577" s="1">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
       <c r="C577" s="1">
         <v>11.0</v>
@@ -14669,10 +14669,10 @@
     </row>
     <row r="578">
       <c r="A578" s="1">
-        <v>669.0</v>
+        <v>670.0</v>
       </c>
       <c r="B578" s="1">
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
       <c r="C578" s="1">
         <v>11.0</v>
@@ -14683,10 +14683,10 @@
     </row>
     <row r="579">
       <c r="A579" s="1">
-        <v>670.0</v>
+        <v>671.0</v>
       </c>
       <c r="B579" s="1">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="C579" s="1">
         <v>11.0</v>
@@ -14697,10 +14697,10 @@
     </row>
     <row r="580">
       <c r="A580" s="1">
-        <v>671.0</v>
+        <v>672.0</v>
       </c>
       <c r="B580" s="1">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
       <c r="C580" s="1">
         <v>11.0</v>
@@ -14711,10 +14711,10 @@
     </row>
     <row r="581">
       <c r="A581" s="1">
-        <v>672.0</v>
+        <v>673.0</v>
       </c>
       <c r="B581" s="1">
-        <v>33.0</v>
+        <v>34.0</v>
       </c>
       <c r="C581" s="1">
         <v>11.0</v>
@@ -14725,10 +14725,10 @@
     </row>
     <row r="582">
       <c r="A582" s="1">
-        <v>673.0</v>
+        <v>674.0</v>
       </c>
       <c r="B582" s="1">
-        <v>34.0</v>
+        <v>35.0</v>
       </c>
       <c r="C582" s="1">
         <v>11.0</v>
@@ -14739,10 +14739,10 @@
     </row>
     <row r="583">
       <c r="A583" s="1">
-        <v>674.0</v>
+        <v>675.0</v>
       </c>
       <c r="B583" s="1">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
       <c r="C583" s="1">
         <v>11.0</v>
@@ -14753,10 +14753,10 @@
     </row>
     <row r="584">
       <c r="A584" s="1">
-        <v>675.0</v>
+        <v>676.0</v>
       </c>
       <c r="B584" s="1">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="C584" s="1">
         <v>11.0</v>
@@ -14767,10 +14767,10 @@
     </row>
     <row r="585">
       <c r="A585" s="1">
-        <v>676.0</v>
+        <v>677.0</v>
       </c>
       <c r="B585" s="1">
-        <v>37.0</v>
+        <v>38.0</v>
       </c>
       <c r="C585" s="1">
         <v>11.0</v>
@@ -14781,10 +14781,10 @@
     </row>
     <row r="586">
       <c r="A586" s="1">
-        <v>677.0</v>
+        <v>678.0</v>
       </c>
       <c r="B586" s="1">
-        <v>38.0</v>
+        <v>40.0</v>
       </c>
       <c r="C586" s="1">
         <v>11.0</v>
@@ -14795,10 +14795,10 @@
     </row>
     <row r="587">
       <c r="A587" s="1">
-        <v>678.0</v>
+        <v>679.0</v>
       </c>
       <c r="B587" s="1">
-        <v>40.0</v>
+        <v>41.0</v>
       </c>
       <c r="C587" s="1">
         <v>11.0</v>
@@ -14809,10 +14809,10 @@
     </row>
     <row r="588">
       <c r="A588" s="1">
-        <v>679.0</v>
+        <v>680.0</v>
       </c>
       <c r="B588" s="1">
-        <v>41.0</v>
+        <v>42.0</v>
       </c>
       <c r="C588" s="1">
         <v>11.0</v>
@@ -14820,30 +14820,33 @@
       <c r="D588" s="1">
         <v>1.0</v>
       </c>
+      <c r="E588" s="1" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="589">
       <c r="A589" s="1">
-        <v>680.0</v>
+        <v>681.0</v>
       </c>
       <c r="B589" s="1">
-        <v>42.0</v>
+        <v>63.0</v>
       </c>
       <c r="C589" s="1">
         <v>11.0</v>
       </c>
       <c r="D589" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E589" s="1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="1">
-        <v>681.0</v>
+        <v>682.0</v>
       </c>
       <c r="B590" s="1">
-        <v>63.0</v>
+        <v>64.0</v>
       </c>
       <c r="C590" s="1">
         <v>11.0</v>
@@ -14851,16 +14854,13 @@
       <c r="D590" s="1">
         <v>2.0</v>
       </c>
-      <c r="E590" s="1" t="s">
-        <v>426</v>
-      </c>
     </row>
     <row r="591">
       <c r="A591" s="1">
-        <v>682.0</v>
+        <v>683.0</v>
       </c>
       <c r="B591" s="1">
-        <v>64.0</v>
+        <v>65.0</v>
       </c>
       <c r="C591" s="1">
         <v>11.0</v>
@@ -14871,10 +14871,10 @@
     </row>
     <row r="592">
       <c r="A592" s="1">
-        <v>683.0</v>
+        <v>684.0</v>
       </c>
       <c r="B592" s="1">
-        <v>65.0</v>
+        <v>111.0</v>
       </c>
       <c r="C592" s="1">
         <v>11.0</v>
@@ -14885,10 +14885,10 @@
     </row>
     <row r="593">
       <c r="A593" s="1">
-        <v>684.0</v>
+        <v>685.0</v>
       </c>
       <c r="B593" s="1">
-        <v>111.0</v>
+        <v>66.0</v>
       </c>
       <c r="C593" s="1">
         <v>11.0</v>
@@ -14896,13 +14896,16 @@
       <c r="D593" s="1">
         <v>2.0</v>
       </c>
+      <c r="E593" s="1" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="594">
       <c r="A594" s="1">
-        <v>685.0</v>
+        <v>686.0</v>
       </c>
       <c r="B594" s="1">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
       <c r="C594" s="1">
         <v>11.0</v>
@@ -14910,30 +14913,27 @@
       <c r="D594" s="1">
         <v>2.0</v>
       </c>
-      <c r="E594" s="1" t="s">
-        <v>427</v>
-      </c>
     </row>
     <row r="595">
       <c r="A595" s="1">
-        <v>686.0</v>
+        <v>687.0</v>
       </c>
       <c r="B595" s="1">
-        <v>67.0</v>
+        <v>1.0</v>
       </c>
       <c r="C595" s="1">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="D595" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="1">
-        <v>687.0</v>
+        <v>688.0</v>
       </c>
       <c r="B596" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C596" s="1">
         <v>12.0</v>
@@ -14944,10 +14944,10 @@
     </row>
     <row r="597">
       <c r="A597" s="1">
-        <v>688.0</v>
+        <v>689.0</v>
       </c>
       <c r="B597" s="1">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="C597" s="1">
         <v>12.0</v>
@@ -14958,10 +14958,10 @@
     </row>
     <row r="598">
       <c r="A598" s="1">
-        <v>689.0</v>
+        <v>690.0</v>
       </c>
       <c r="B598" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C598" s="1">
         <v>12.0</v>
@@ -14972,10 +14972,10 @@
     </row>
     <row r="599">
       <c r="A599" s="1">
-        <v>690.0</v>
+        <v>691.0</v>
       </c>
       <c r="B599" s="1">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C599" s="1">
         <v>12.0</v>
@@ -14986,10 +14986,10 @@
     </row>
     <row r="600">
       <c r="A600" s="1">
-        <v>691.0</v>
+        <v>692.0</v>
       </c>
       <c r="B600" s="1">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="C600" s="1">
         <v>12.0</v>
@@ -15000,10 +15000,10 @@
     </row>
     <row r="601">
       <c r="A601" s="1">
-        <v>692.0</v>
+        <v>693.0</v>
       </c>
       <c r="B601" s="1">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="C601" s="1">
         <v>12.0</v>
@@ -15014,10 +15014,10 @@
     </row>
     <row r="602">
       <c r="A602" s="1">
-        <v>693.0</v>
+        <v>694.0</v>
       </c>
       <c r="B602" s="1">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="C602" s="1">
         <v>12.0</v>
@@ -15028,10 +15028,10 @@
     </row>
     <row r="603">
       <c r="A603" s="1">
-        <v>694.0</v>
+        <v>695.0</v>
       </c>
       <c r="B603" s="1">
-        <v>8.0</v>
+        <v>9.0</v>
       </c>
       <c r="C603" s="1">
         <v>12.0</v>
@@ -15042,10 +15042,10 @@
     </row>
     <row r="604">
       <c r="A604" s="1">
-        <v>695.0</v>
+        <v>696.0</v>
       </c>
       <c r="B604" s="1">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
       <c r="C604" s="1">
         <v>12.0</v>
@@ -15056,10 +15056,10 @@
     </row>
     <row r="605">
       <c r="A605" s="1">
-        <v>696.0</v>
+        <v>697.0</v>
       </c>
       <c r="B605" s="1">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
       <c r="C605" s="1">
         <v>12.0</v>
@@ -15070,10 +15070,10 @@
     </row>
     <row r="606">
       <c r="A606" s="1">
-        <v>697.0</v>
+        <v>698.0</v>
       </c>
       <c r="B606" s="1">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="C606" s="1">
         <v>12.0</v>
@@ -15084,10 +15084,10 @@
     </row>
     <row r="607">
       <c r="A607" s="1">
-        <v>698.0</v>
+        <v>699.0</v>
       </c>
       <c r="B607" s="1">
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="C607" s="1">
         <v>12.0</v>
@@ -15098,10 +15098,10 @@
     </row>
     <row r="608">
       <c r="A608" s="1">
-        <v>699.0</v>
+        <v>700.0</v>
       </c>
       <c r="B608" s="1">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
       <c r="C608" s="1">
         <v>12.0</v>
@@ -15112,10 +15112,10 @@
     </row>
     <row r="609">
       <c r="A609" s="1">
-        <v>700.0</v>
+        <v>701.0</v>
       </c>
       <c r="B609" s="1">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="C609" s="1">
         <v>12.0</v>
@@ -15126,10 +15126,10 @@
     </row>
     <row r="610">
       <c r="A610" s="1">
-        <v>701.0</v>
+        <v>702.0</v>
       </c>
       <c r="B610" s="1">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C610" s="1">
         <v>12.0</v>
@@ -15140,10 +15140,10 @@
     </row>
     <row r="611">
       <c r="A611" s="1">
-        <v>702.0</v>
+        <v>703.0</v>
       </c>
       <c r="B611" s="1">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
       <c r="C611" s="1">
         <v>12.0</v>
@@ -15154,10 +15154,10 @@
     </row>
     <row r="612">
       <c r="A612" s="1">
-        <v>703.0</v>
+        <v>704.0</v>
       </c>
       <c r="B612" s="1">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
       <c r="C612" s="1">
         <v>12.0</v>
@@ -15168,10 +15168,10 @@
     </row>
     <row r="613">
       <c r="A613" s="1">
-        <v>704.0</v>
+        <v>705.0</v>
       </c>
       <c r="B613" s="1">
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="C613" s="1">
         <v>12.0</v>
@@ -15182,10 +15182,10 @@
     </row>
     <row r="614">
       <c r="A614" s="1">
-        <v>705.0</v>
+        <v>706.0</v>
       </c>
       <c r="B614" s="1">
-        <v>19.0</v>
+        <v>20.0</v>
       </c>
       <c r="C614" s="1">
         <v>12.0</v>
@@ -15196,10 +15196,10 @@
     </row>
     <row r="615">
       <c r="A615" s="1">
-        <v>706.0</v>
+        <v>707.0</v>
       </c>
       <c r="B615" s="1">
-        <v>20.0</v>
+        <v>21.0</v>
       </c>
       <c r="C615" s="1">
         <v>12.0</v>
@@ -15210,10 +15210,10 @@
     </row>
     <row r="616">
       <c r="A616" s="1">
-        <v>707.0</v>
+        <v>708.0</v>
       </c>
       <c r="B616" s="1">
-        <v>21.0</v>
+        <v>22.0</v>
       </c>
       <c r="C616" s="1">
         <v>12.0</v>
@@ -15224,10 +15224,10 @@
     </row>
     <row r="617">
       <c r="A617" s="1">
-        <v>708.0</v>
+        <v>709.0</v>
       </c>
       <c r="B617" s="1">
-        <v>22.0</v>
+        <v>23.0</v>
       </c>
       <c r="C617" s="1">
         <v>12.0</v>
@@ -15238,10 +15238,10 @@
     </row>
     <row r="618">
       <c r="A618" s="1">
-        <v>709.0</v>
+        <v>710.0</v>
       </c>
       <c r="B618" s="1">
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="C618" s="1">
         <v>12.0</v>
@@ -15252,10 +15252,10 @@
     </row>
     <row r="619">
       <c r="A619" s="1">
-        <v>710.0</v>
+        <v>711.0</v>
       </c>
       <c r="B619" s="1">
-        <v>24.0</v>
+        <v>25.0</v>
       </c>
       <c r="C619" s="1">
         <v>12.0</v>
@@ -15266,10 +15266,10 @@
     </row>
     <row r="620">
       <c r="A620" s="1">
-        <v>711.0</v>
+        <v>712.0</v>
       </c>
       <c r="B620" s="1">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="C620" s="1">
         <v>12.0</v>
@@ -15280,10 +15280,10 @@
     </row>
     <row r="621">
       <c r="A621" s="1">
-        <v>712.0</v>
+        <v>713.0</v>
       </c>
       <c r="B621" s="1">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
       <c r="C621" s="1">
         <v>12.0</v>
@@ -15294,10 +15294,10 @@
     </row>
     <row r="622">
       <c r="A622" s="1">
-        <v>713.0</v>
+        <v>714.0</v>
       </c>
       <c r="B622" s="1">
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
       <c r="C622" s="1">
         <v>12.0</v>
@@ -15308,10 +15308,10 @@
     </row>
     <row r="623">
       <c r="A623" s="1">
-        <v>714.0</v>
+        <v>715.0</v>
       </c>
       <c r="B623" s="1">
-        <v>28.0</v>
+        <v>110.0</v>
       </c>
       <c r="C623" s="1">
         <v>12.0</v>
@@ -15322,10 +15322,10 @@
     </row>
     <row r="624">
       <c r="A624" s="1">
-        <v>715.0</v>
+        <v>716.0</v>
       </c>
       <c r="B624" s="1">
-        <v>110.0</v>
+        <v>29.0</v>
       </c>
       <c r="C624" s="1">
         <v>12.0</v>
@@ -15336,10 +15336,10 @@
     </row>
     <row r="625">
       <c r="A625" s="1">
-        <v>716.0</v>
+        <v>717.0</v>
       </c>
       <c r="B625" s="1">
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
       <c r="C625" s="1">
         <v>12.0</v>
@@ -15350,10 +15350,10 @@
     </row>
     <row r="626">
       <c r="A626" s="1">
-        <v>717.0</v>
+        <v>718.0</v>
       </c>
       <c r="B626" s="1">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="C626" s="1">
         <v>12.0</v>
@@ -15364,10 +15364,10 @@
     </row>
     <row r="627">
       <c r="A627" s="1">
-        <v>718.0</v>
+        <v>719.0</v>
       </c>
       <c r="B627" s="1">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
       <c r="C627" s="1">
         <v>12.0</v>
@@ -15378,10 +15378,10 @@
     </row>
     <row r="628">
       <c r="A628" s="1">
-        <v>719.0</v>
+        <v>720.0</v>
       </c>
       <c r="B628" s="1">
-        <v>33.0</v>
+        <v>34.0</v>
       </c>
       <c r="C628" s="1">
         <v>12.0</v>
@@ -15392,10 +15392,10 @@
     </row>
     <row r="629">
       <c r="A629" s="1">
-        <v>720.0</v>
+        <v>721.0</v>
       </c>
       <c r="B629" s="1">
-        <v>34.0</v>
+        <v>35.0</v>
       </c>
       <c r="C629" s="1">
         <v>12.0</v>
@@ -15406,10 +15406,10 @@
     </row>
     <row r="630">
       <c r="A630" s="1">
-        <v>721.0</v>
+        <v>722.0</v>
       </c>
       <c r="B630" s="1">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
       <c r="C630" s="1">
         <v>12.0</v>
@@ -15420,10 +15420,10 @@
     </row>
     <row r="631">
       <c r="A631" s="1">
-        <v>722.0</v>
+        <v>723.0</v>
       </c>
       <c r="B631" s="1">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="C631" s="1">
         <v>12.0</v>
@@ -15434,10 +15434,10 @@
     </row>
     <row r="632">
       <c r="A632" s="1">
-        <v>723.0</v>
+        <v>724.0</v>
       </c>
       <c r="B632" s="1">
-        <v>37.0</v>
+        <v>38.0</v>
       </c>
       <c r="C632" s="1">
         <v>12.0</v>
@@ -15448,10 +15448,10 @@
     </row>
     <row r="633">
       <c r="A633" s="1">
-        <v>724.0</v>
+        <v>725.0</v>
       </c>
       <c r="B633" s="1">
-        <v>38.0</v>
+        <v>40.0</v>
       </c>
       <c r="C633" s="1">
         <v>12.0</v>
@@ -15462,10 +15462,10 @@
     </row>
     <row r="634">
       <c r="A634" s="1">
-        <v>725.0</v>
+        <v>726.0</v>
       </c>
       <c r="B634" s="1">
-        <v>40.0</v>
+        <v>41.0</v>
       </c>
       <c r="C634" s="1">
         <v>12.0</v>
@@ -15476,10 +15476,10 @@
     </row>
     <row r="635">
       <c r="A635" s="1">
-        <v>726.0</v>
+        <v>727.0</v>
       </c>
       <c r="B635" s="1">
-        <v>41.0</v>
+        <v>42.0</v>
       </c>
       <c r="C635" s="1">
         <v>12.0</v>
@@ -15487,13 +15487,16 @@
       <c r="D635" s="1">
         <v>1.0</v>
       </c>
+      <c r="E635" s="1" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="636">
       <c r="A636" s="1">
-        <v>727.0</v>
+        <v>728.0</v>
       </c>
       <c r="B636" s="1">
-        <v>42.0</v>
+        <v>63.0</v>
       </c>
       <c r="C636" s="1">
         <v>12.0</v>
@@ -15502,15 +15505,15 @@
         <v>1.0</v>
       </c>
       <c r="E636" s="1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="1">
-        <v>728.0</v>
+        <v>729.0</v>
       </c>
       <c r="B637" s="1">
-        <v>63.0</v>
+        <v>64.0</v>
       </c>
       <c r="C637" s="1">
         <v>12.0</v>
@@ -15518,16 +15521,13 @@
       <c r="D637" s="1">
         <v>1.0</v>
       </c>
-      <c r="E637" s="1" t="s">
-        <v>426</v>
-      </c>
     </row>
     <row r="638">
       <c r="A638" s="1">
-        <v>729.0</v>
+        <v>730.0</v>
       </c>
       <c r="B638" s="1">
-        <v>64.0</v>
+        <v>66.0</v>
       </c>
       <c r="C638" s="1">
         <v>12.0</v>
@@ -15535,19 +15535,22 @@
       <c r="D638" s="1">
         <v>1.0</v>
       </c>
+      <c r="E638" s="1" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="639">
       <c r="A639" s="1">
-        <v>730.0</v>
+        <v>731.0</v>
       </c>
       <c r="B639" s="1">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
       <c r="C639" s="1">
         <v>12.0</v>
       </c>
       <c r="D639" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E639" s="1" t="s">
         <v>427</v>
@@ -15555,10 +15558,10 @@
     </row>
     <row r="640">
       <c r="A640" s="1">
-        <v>731.0</v>
+        <v>732.0</v>
       </c>
       <c r="B640" s="1">
-        <v>67.0</v>
+        <v>74.0</v>
       </c>
       <c r="C640" s="1">
         <v>12.0</v>
@@ -15567,15 +15570,15 @@
         <v>2.0</v>
       </c>
       <c r="E640" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="1">
-        <v>732.0</v>
+        <v>733.0</v>
       </c>
       <c r="B641" s="1">
-        <v>74.0</v>
+        <v>76.0</v>
       </c>
       <c r="C641" s="1">
         <v>12.0</v>
@@ -15589,10 +15592,10 @@
     </row>
     <row r="642">
       <c r="A642" s="1">
-        <v>733.0</v>
+        <v>734.0</v>
       </c>
       <c r="B642" s="1">
-        <v>76.0</v>
+        <v>78.0</v>
       </c>
       <c r="C642" s="1">
         <v>12.0</v>
@@ -15606,10 +15609,10 @@
     </row>
     <row r="643">
       <c r="A643" s="1">
-        <v>734.0</v>
+        <v>735.0</v>
       </c>
       <c r="B643" s="1">
-        <v>78.0</v>
+        <v>80.0</v>
       </c>
       <c r="C643" s="1">
         <v>12.0</v>
@@ -15622,21 +15625,8 @@
       </c>
     </row>
     <row r="644">
-      <c r="A644" s="1">
-        <v>735.0</v>
-      </c>
-      <c r="B644" s="1">
-        <v>80.0</v>
-      </c>
-      <c r="C644" s="1">
-        <v>12.0</v>
-      </c>
-      <c r="D644" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="E644" s="1" t="s">
-        <v>428</v>
-      </c>
+      <c r="B644" s="1"/>
+      <c r="D644" s="1"/>
     </row>
     <row r="645">
       <c r="B645" s="1"/>
@@ -19589,10 +19579,6 @@
     <row r="1632">
       <c r="B1632" s="1"/>
       <c r="D1632" s="1"/>
-    </row>
-    <row r="1633">
-      <c r="B1633" s="1"/>
-      <c r="D1633" s="1"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
added aliases for procedure 112 - 115 and changed global rules to fetch internalNotes
</commit_message>
<xml_diff>
--- a/procedure_lookup_project.xlsx
+++ b/procedure_lookup_project.xlsx
@@ -19,14 +19,15 @@
   <definedNames>
     <definedName hidden="1" localSheetId="6" name="_xlnm._FilterDatabase">ProcedureClinics!$A$1:$F$1185</definedName>
     <definedName hidden="1" localSheetId="7" name="_xlnm._FilterDatabase">ProcedureRadiologists!$A$1:$E$2271</definedName>
-    <definedName hidden="1" localSheetId="8" name="_xlnm._FilterDatabase">ProcedureBookingCategories!$A$1:$F$1539</definedName>
+    <definedName hidden="1" localSheetId="8" name="_xlnm._FilterDatabase">ProcedureBookingCategories!$A$1:$F$1540</definedName>
+    <definedName hidden="1" localSheetId="10" name="_xlnm._FilterDatabase">ProcedureAliases!$A$1:$D$360</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4433" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4455" uniqueCount="748">
   <si>
     <t>Table</t>
   </si>
@@ -2227,6 +2228,36 @@
     <t>Kneecap Bursa Injection</t>
   </si>
   <si>
+    <t>Any other joint aspiration</t>
+  </si>
+  <si>
+    <t>Joint Aspiration Other</t>
+  </si>
+  <si>
+    <t>Piriformis Botox</t>
+  </si>
+  <si>
+    <t>Piri Botox Injection</t>
+  </si>
+  <si>
+    <t>Botox Injection</t>
+  </si>
+  <si>
+    <t>TMJ Botox Injection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMJ </t>
+  </si>
+  <si>
+    <t>TMJ Migraines</t>
+  </si>
+  <si>
+    <t>Migraine Botox</t>
+  </si>
+  <si>
+    <t>Botox Head ache</t>
+  </si>
+  <si>
     <t>ProcedureRuleID</t>
   </si>
   <si>
@@ -2600,8 +2631,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F1539" displayName="tbProcedureBookingCategories" name="tbProcedureBookingCategories" id="8">
-  <autoFilter ref="$A$1:$F$1539"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F1540" displayName="tbProcedureBookingCategories" name="tbProcedureBookingCategories" id="8">
+  <autoFilter ref="$A$1:$F$1540"/>
   <tableColumns count="6">
     <tableColumn name="ProcedureBookingCategoryID" id="1"/>
     <tableColumn name="ProcedureID" id="2"/>
@@ -2615,7 +2646,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D349" displayName="tbProcedureAliases" name="tbProcedureAliases" id="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D360" displayName="tbProcedureAliases" name="tbProcedureAliases" id="9">
+  <autoFilter ref="$A$1:$D$360"/>
   <tableColumns count="4">
     <tableColumn name="ProcedureAliasID" id="1"/>
     <tableColumn name="ProcedureID" id="2"/>
@@ -7876,6 +7908,160 @@
         <v>489</v>
       </c>
     </row>
+    <row r="350" ht="22.5" customHeight="1">
+      <c r="A350" s="6">
+        <v>349.0</v>
+      </c>
+      <c r="B350" s="6">
+        <v>115.0</v>
+      </c>
+      <c r="C350" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="D350" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="351" ht="22.5" customHeight="1">
+      <c r="A351" s="6">
+        <v>350.0</v>
+      </c>
+      <c r="B351" s="6">
+        <v>115.0</v>
+      </c>
+      <c r="C351" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="D351" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="352" ht="22.5" customHeight="1">
+      <c r="A352" s="6">
+        <v>351.0</v>
+      </c>
+      <c r="B352" s="6">
+        <v>114.0</v>
+      </c>
+      <c r="C352" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="D352" s="6" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="353" ht="22.5" customHeight="1">
+      <c r="A353" s="6">
+        <v>352.0</v>
+      </c>
+      <c r="B353" s="6">
+        <v>114.0</v>
+      </c>
+      <c r="C353" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="D353" s="6" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="354" ht="22.5" customHeight="1">
+      <c r="A354" s="6">
+        <v>353.0</v>
+      </c>
+      <c r="B354" s="6">
+        <v>114.0</v>
+      </c>
+      <c r="C354" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="D354" s="6" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="355" ht="22.5" customHeight="1">
+      <c r="A355" s="6">
+        <v>354.0</v>
+      </c>
+      <c r="B355" s="6">
+        <v>113.0</v>
+      </c>
+      <c r="C355" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="D355" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="356" ht="22.5" customHeight="1">
+      <c r="A356" s="6">
+        <v>355.0</v>
+      </c>
+      <c r="B356" s="6">
+        <v>113.0</v>
+      </c>
+      <c r="C356" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="D356" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="357" ht="22.5" customHeight="1">
+      <c r="A357" s="6">
+        <v>356.0</v>
+      </c>
+      <c r="B357" s="6">
+        <v>113.0</v>
+      </c>
+      <c r="C357" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="D357" s="6" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="358" ht="22.5" customHeight="1">
+      <c r="A358" s="6">
+        <v>357.0</v>
+      </c>
+      <c r="B358" s="6">
+        <v>112.0</v>
+      </c>
+      <c r="C358" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="D358" s="6" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="359" ht="22.5" customHeight="1">
+      <c r="A359" s="6">
+        <v>358.0</v>
+      </c>
+      <c r="B359" s="6">
+        <v>112.0</v>
+      </c>
+      <c r="C359" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D359" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="360" ht="22.5" customHeight="1">
+      <c r="A360" s="6">
+        <v>359.0</v>
+      </c>
+      <c r="B360" s="6">
+        <v>112.0</v>
+      </c>
+      <c r="C360" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="D360" s="6" t="s">
+        <v>708</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A1000">
     <cfRule type="expression" dxfId="5" priority="1">
@@ -7909,22 +8095,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>281</v>
@@ -90908,6 +91094,24 @@
       </c>
       <c r="F1539" s="7"/>
     </row>
+    <row r="1540" ht="22.5" customHeight="1">
+      <c r="A1540" s="6">
+        <v>1635.0</v>
+      </c>
+      <c r="B1540" s="6">
+        <v>46.0</v>
+      </c>
+      <c r="C1540" s="6">
+        <v>33.0</v>
+      </c>
+      <c r="D1540" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="E1540" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F1540" s="7"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A1811 C1527:C1538">
     <cfRule type="expression" dxfId="5" priority="1">

</xml_diff>